<commit_message>
Restore verbatim Asset Register Machine IDs (EX 006, C-HEADT 007, C-HEADT 008) via migration 0011
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/database/Equipment_Register.xlsx
+++ b/database/Equipment_Register.xlsx
@@ -15,7 +15,7 @@
     <t xml:space="preserve">WORKSHOP EQUIPMENT REGISTER — 21 OCTOBER 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated 21/10/2026 12:07 by WMSv2 Recovery  •  116 assets  •  Availability = (operating hours − downtime) ÷ operating hours</t>
+    <t xml:space="preserve">Generated 21/10/2026 17:51 by WMSv2 Recovery  •  116 assets  •  Availability = (operating hours − downtime) ÷ operating hours</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -222,7 +222,7 @@
     <t xml:space="preserve">Bucket Worn out</t>
   </si>
   <si>
-    <t xml:space="preserve">C-HV-EX 006</t>
+    <t xml:space="preserve">EX 006</t>
   </si>
   <si>
     <t xml:space="preserve">XE500</t>
@@ -369,7 +369,7 @@
     <t xml:space="preserve">Engine no start</t>
   </si>
   <si>
-    <t xml:space="preserve">C-HE-ADT 007</t>
+    <t xml:space="preserve">C-HEADT 007</t>
   </si>
   <si>
     <t xml:space="preserve">CAT00745P3F601164</t>
@@ -378,7 +378,7 @@
     <t xml:space="preserve">Differential problem</t>
   </si>
   <si>
-    <t xml:space="preserve">C-HE-ADT 008</t>
+    <t xml:space="preserve">C-HEADT 008</t>
   </si>
   <si>
     <t xml:space="preserve">CAT00745V3F601199</t>
@@ -1257,7 +1257,7 @@
     <t xml:space="preserve">  existing value.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Generated 21/10/2026 12:07.</t>
+    <t xml:space="preserve">• Generated 21/10/2026 17:51.</t>
   </si>
 </sst>
 </file>

</xml_diff>